<commit_message>
feat: update autho model update
</commit_message>
<xml_diff>
--- a/backend/exports/vendors.xlsx
+++ b/backend/exports/vendors.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="65">
   <si>
     <t>Company Name</t>
   </si>
@@ -32,6 +32,39 @@
   </si>
   <si>
     <t>Registered On</t>
+  </si>
+  <si>
+    <t>golden</t>
+  </si>
+  <si>
+    <t>33AAACH7409R1Z8</t>
+  </si>
+  <si>
+    <t>tamil</t>
+  </si>
+  <si>
+    <t>toy</t>
+  </si>
+  <si>
+    <t>8545956525</t>
+  </si>
+  <si>
+    <t>abhishek@yahoomail.com</t>
+  </si>
+  <si>
+    <t>30/9/2026, 3:25:41 pm</t>
+  </si>
+  <si>
+    <t>tamil nadu</t>
+  </si>
+  <si>
+    <t>8545965255</t>
+  </si>
+  <si>
+    <t>golden4521@gmail.com</t>
+  </si>
+  <si>
+    <t>30/9/2026, 3:24:42 pm</t>
   </si>
   <si>
     <t>jhdhfj</t>
@@ -553,7 +586,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -613,163 +646,209 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" t="s">
         <v>14</v>
       </c>
-      <c r="B3" t="s">
+      <c r="D3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" t="s">
         <v>15</v>
       </c>
-      <c r="C3" t="s">
+      <c r="F3" t="s">
         <v>16</v>
       </c>
-      <c r="D3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E3" t="s">
+      <c r="G3" t="s">
         <v>17</v>
-      </c>
-      <c r="F3" t="s">
-        <v>18</v>
-      </c>
-      <c r="G3" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" t="s">
         <v>20</v>
       </c>
-      <c r="B4" t="s">
+      <c r="D4" t="s">
         <v>21</v>
       </c>
-      <c r="C4" t="s">
+      <c r="E4" t="s">
         <v>22</v>
       </c>
-      <c r="D4" t="s">
+      <c r="F4" t="s">
         <v>23</v>
       </c>
-      <c r="E4" t="s">
+      <c r="G4" t="s">
         <v>24</v>
-      </c>
-      <c r="F4" t="s">
-        <v>25</v>
-      </c>
-      <c r="G4" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" t="s">
         <v>27</v>
       </c>
-      <c r="B5" t="s">
+      <c r="D5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E5" t="s">
         <v>28</v>
       </c>
-      <c r="C5" t="s">
-        <v>22</v>
-      </c>
-      <c r="D5" t="s">
+      <c r="F5" t="s">
         <v>29</v>
       </c>
-      <c r="E5" t="s">
+      <c r="G5" t="s">
         <v>30</v>
-      </c>
-      <c r="F5" t="s">
-        <v>31</v>
-      </c>
-      <c r="G5" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" t="s">
         <v>33</v>
       </c>
-      <c r="B6" t="s">
+      <c r="D6" t="s">
         <v>34</v>
       </c>
-      <c r="C6" t="s">
+      <c r="E6" t="s">
         <v>35</v>
       </c>
-      <c r="D6" t="s">
+      <c r="F6" t="s">
         <v>36</v>
       </c>
-      <c r="E6" t="s">
+      <c r="G6" t="s">
         <v>37</v>
-      </c>
-      <c r="F6" t="s">
-        <v>38</v>
-      </c>
-      <c r="G6" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="B7" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="C7" t="s">
+        <v>33</v>
+      </c>
+      <c r="D7" t="s">
         <v>40</v>
       </c>
-      <c r="D7" t="s">
-        <v>29</v>
-      </c>
       <c r="E7" t="s">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c r="F7" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B8" t="s">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="C8" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D8" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E8" t="s">
-        <v>30</v>
+        <v>48</v>
       </c>
       <c r="F8" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="G8" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="B9" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="C9" t="s">
+        <v>51</v>
+      </c>
+      <c r="D9" t="s">
         <v>40</v>
       </c>
-      <c r="D9" t="s">
-        <v>50</v>
-      </c>
       <c r="E9" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="F9" t="s">
         <v>52</v>
       </c>
       <c r="G9" t="s">
         <v>53</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>54</v>
+      </c>
+      <c r="B10" t="s">
+        <v>39</v>
+      </c>
+      <c r="C10" t="s">
+        <v>55</v>
+      </c>
+      <c r="D10" t="s">
+        <v>56</v>
+      </c>
+      <c r="E10" t="s">
+        <v>41</v>
+      </c>
+      <c r="F10" t="s">
+        <v>57</v>
+      </c>
+      <c r="G10" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>59</v>
+      </c>
+      <c r="B11" t="s">
+        <v>60</v>
+      </c>
+      <c r="C11" t="s">
+        <v>51</v>
+      </c>
+      <c r="D11" t="s">
+        <v>61</v>
+      </c>
+      <c r="E11" t="s">
+        <v>62</v>
+      </c>
+      <c r="F11" t="s">
+        <v>63</v>
+      </c>
+      <c r="G11" t="s">
+        <v>64</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: update - service  date 3-oct-26 8th commit
</commit_message>
<xml_diff>
--- a/backend/exports/vendors.xlsx
+++ b/backend/exports/vendors.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="86">
   <si>
     <t>Company Name</t>
   </si>
@@ -32,6 +32,69 @@
   </si>
   <si>
     <t>Registered On</t>
+  </si>
+  <si>
+    <t>vendar1</t>
+  </si>
+  <si>
+    <t>27AAAAP0267H2ZN</t>
+  </si>
+  <si>
+    <t>fake</t>
+  </si>
+  <si>
+    <t>demo</t>
+  </si>
+  <si>
+    <t>2536253623</t>
+  </si>
+  <si>
+    <t>vendar1@gmail.com</t>
+  </si>
+  <si>
+    <t>7/10/2026, 3:20:12 pm</t>
+  </si>
+  <si>
+    <t>fhhgfh</t>
+  </si>
+  <si>
+    <t>30AAAAP0267H1Z1</t>
+  </si>
+  <si>
+    <t>demo 1</t>
+  </si>
+  <si>
+    <t>demo 2</t>
+  </si>
+  <si>
+    <t>8569636564</t>
+  </si>
+  <si>
+    <t>demo56@gmail.com</t>
+  </si>
+  <si>
+    <t>6/10/2026, 1:31:55 pm</t>
+  </si>
+  <si>
+    <t>waewfe</t>
+  </si>
+  <si>
+    <t>33AAFCC9980MZZ4</t>
+  </si>
+  <si>
+    <t>demo data</t>
+  </si>
+  <si>
+    <t>demo data 2</t>
+  </si>
+  <si>
+    <t>5236525252</t>
+  </si>
+  <si>
+    <t>demo25@gmail.com</t>
+  </si>
+  <si>
+    <t>6/10/2026, 1:30:42 pm</t>
   </si>
   <si>
     <t>golden</t>
@@ -586,7 +649,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -646,209 +709,278 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="B3" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="C3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D3" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="E3" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="F3" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="G3" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C4" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D4" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="E4" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F4" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="G4" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="B5" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C5" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="D5" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="E5" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="F5" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="G5" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" t="s">
+        <v>35</v>
+      </c>
+      <c r="D6" t="s">
         <v>31</v>
       </c>
-      <c r="B6" t="s">
-        <v>32</v>
-      </c>
-      <c r="C6" t="s">
-        <v>33</v>
-      </c>
-      <c r="D6" t="s">
-        <v>34</v>
-      </c>
       <c r="E6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B7" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C7" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="D7" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E7" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F7" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G7" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B8" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C8" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D8" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G8" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>38</v>
+        <v>52</v>
       </c>
       <c r="B9" t="s">
-        <v>39</v>
+        <v>53</v>
       </c>
       <c r="C9" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="D9" t="s">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="E9" t="s">
-        <v>41</v>
+        <v>56</v>
       </c>
       <c r="F9" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="G9" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>59</v>
+      </c>
+      <c r="B10" t="s">
+        <v>60</v>
+      </c>
+      <c r="C10" t="s">
         <v>54</v>
       </c>
-      <c r="B10" t="s">
-        <v>39</v>
-      </c>
-      <c r="C10" t="s">
-        <v>55</v>
-      </c>
       <c r="D10" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="E10" t="s">
-        <v>41</v>
+        <v>62</v>
       </c>
       <c r="F10" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="G10" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>65</v>
+      </c>
+      <c r="B11" t="s">
+        <v>66</v>
+      </c>
+      <c r="C11" t="s">
+        <v>67</v>
+      </c>
+      <c r="D11" t="s">
+        <v>68</v>
+      </c>
+      <c r="E11" t="s">
+        <v>69</v>
+      </c>
+      <c r="F11" t="s">
+        <v>70</v>
+      </c>
+      <c r="G11" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>59</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B12" t="s">
         <v>60</v>
       </c>
-      <c r="C11" t="s">
-        <v>51</v>
-      </c>
-      <c r="D11" t="s">
+      <c r="C12" t="s">
+        <v>72</v>
+      </c>
+      <c r="D12" t="s">
         <v>61</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E12" t="s">
         <v>62</v>
       </c>
-      <c r="F11" t="s">
-        <v>63</v>
-      </c>
-      <c r="G11" t="s">
-        <v>64</v>
+      <c r="F12" t="s">
+        <v>73</v>
+      </c>
+      <c r="G12" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>75</v>
+      </c>
+      <c r="B13" t="s">
+        <v>60</v>
+      </c>
+      <c r="C13" t="s">
+        <v>76</v>
+      </c>
+      <c r="D13" t="s">
+        <v>77</v>
+      </c>
+      <c r="E13" t="s">
+        <v>62</v>
+      </c>
+      <c r="F13" t="s">
+        <v>78</v>
+      </c>
+      <c r="G13" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>80</v>
+      </c>
+      <c r="B14" t="s">
+        <v>81</v>
+      </c>
+      <c r="C14" t="s">
+        <v>72</v>
+      </c>
+      <c r="D14" t="s">
+        <v>82</v>
+      </c>
+      <c r="E14" t="s">
+        <v>83</v>
+      </c>
+      <c r="F14" t="s">
+        <v>84</v>
+      </c>
+      <c r="G14" t="s">
+        <v>85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>